<commit_message>
Prosanitas aggiunta TC tipologia LAB
Nuova tipologia documentale (LAB) per il medesimo software AUTOLABNET 1.1
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#PROSANITASSRLXX/PROSANITASSRL/AUTOLABNET/1.1/report-checklist.xlsx
+++ b/GATEWAY/A1#111#PROSANITASSRLXX/PROSANITASSRL/AUTOLABNET/1.1/report-checklist.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\git_fse\klaus-it-fse-accreditamento\GATEWAY\A1#111#PROSANITASSRLXX\PROSANITASSRL\AUTOLABNET\1.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\git_fse\it-fse-accreditamento\GATEWAY\A1#111#PROSANITASSRLXX\PROSANITASSRL\AUTOLABNET\1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0AB018-A1A6-49FC-919E-0F31F432B735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D7668A-049B-40D4-9D8E-59A8F89ECA6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1425" yWindow="375" windowWidth="23835" windowHeight="14760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Summary!$A$1:$G$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TestCases!$A$9:$W$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">TestCases!$A$9:$W$49</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="688" uniqueCount="284">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -892,6 +892,243 @@
   </si>
   <si>
     <t>2.16.840.1.113883.2.9.2.120.4.4.82a1bcb3ceea777f60fd153f6ec968824d48cbdd877242dfde81a97ed7d9e51f.ee44a54cbf^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+Il Documento CDA2 Laboratorio dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 4" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.
+</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_TOKEN_JWT_LAB_KO</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_TOKEN_JWT_CAMPO_LAB_KO</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_LAB_TIMEOUT</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT7_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori semantici sui Dati (status code 422), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 7" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT9_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori semantici sui Dati (status code 422), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 9" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT10_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori semantici sui Dati (status code 422), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 10" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT11_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 11" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT13_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori sintattici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 13" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT14_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori semantici sui Dati (status code 422), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 14" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT15_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori semantici sui Dati (status code 422), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 15" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT16_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation"al fine di testare la gestione degli errori semantici sui Dati (status code 422), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 16" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_TRASF_CT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+Il Documento CDA2 Laboratorio dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST- OK" riportata nei documenti "Caso di test - Trasfusionale" e "CDA2_Trasfusionale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.
+</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_TRASF_CT2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+Il Documento CDA2 Laboratorio dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST OK - HLA" riportata nei documenti "Caso di test - Trasfusionale" e "CDA2_Trasfusionale_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.
+</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation", al fine di una futura pubblicazione, con esito positivo (status code 201), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+Il Documento CDA2 Laboratorio dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 17" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.
+</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT18</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori sintattici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 18" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO.xlsx" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>VALIDAZIONE_CDA2_LAB_CT19_KO</t>
+  </si>
+  <si>
+    <t>Viene richiamato il servizio di validazione "https://&lt;HOST&gt;:&lt;PORT&gt;/v&lt;major&gt;/documents/validation" al fine di testare la gestione degli errori terminologici sui Dati (status code 400), secondo quanto descritto in https://github.com/ministero-salute/it-fse-support/tree/main/doc/integrazione-gateway.
+I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto nella sezione "CASO DI TEST 19" riportata nei documenti "casi di test LAB" e "CDA2_Referto Medicina di Laboratorio_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
+  </si>
+  <si>
+    <t>4b4c8088d7f7ea7f1b2c6aeb106a5031</t>
+  </si>
+  <si>
+    <t>2026-07-31T23:29:57Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.7a8af6aa7044023ec038bd95b1fe4c0d3018c0328514b38734963865a0a2248f.73411e8321^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-07-31T23:41:13Z</t>
+  </si>
+  <si>
+    <t>578368a6d906ae484bfdce2138e6e240</t>
+  </si>
+  <si>
+    <t>2026-07-31T23:49:09Z</t>
+  </si>
+  <si>
+    <t>1099846fa353f55bd42c7a948f16f3c1</t>
+  </si>
+  <si>
+    <t>2026-07-31T23:51:32Z</t>
+  </si>
+  <si>
+    <t>2026-08-01T00:07:47Z</t>
+  </si>
+  <si>
+    <t>b9919ec60347dfe14cd77ddee064d9a0</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.8d0a2bffa4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>4ab4e9815fb8322757688fecd1e53172</t>
+  </si>
+  <si>
+    <t>2026-08-01T00:16:23Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.29ddd2fc87^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>a35cc52f18734193a3c70494da178f38</t>
+  </si>
+  <si>
+    <t>2026-08-01T22:12:03Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.9f47d92c69^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>9f5b8a5efeac5540babf8c948fda896b</t>
+  </si>
+  <si>
+    <t>2026-08-01T23:07:38Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.6416705fe7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>81ab05993bb3d485be67d8605d69d2ba</t>
+  </si>
+  <si>
+    <t>2026-08-01T23:25:13Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.8e0e155ab6^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>a10c2e1c09875b20ef164d124429c48c</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.14b9996690^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-08-01T23:38:41Z</t>
+  </si>
+  <si>
+    <t>dc2aef502998a1fb05d6f828113054fc</t>
+  </si>
+  <si>
+    <t>2026-08-01T23:52:39Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.de1b59ce39^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>4183713a1038b2e790f6be2d55d45114</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.dbbacc8f43^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-08-02T00:02:10Z</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.737cbfc730^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>1e6773123962e743b408b7c8cae76a36</t>
+  </si>
+  <si>
+    <t>2026-08-02T00:08:28Z</t>
+  </si>
+  <si>
+    <t>09f669816bbe633e80a5102c551bbec2</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.2e0bbc52e6ca77eca20ae80551909a7800addd541f67f905dde03ee582d90171.d972664359^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>2026-08-02T00:31:43Z</t>
+  </si>
+  <si>
+    <t>2026-08-02T00:42:41Z</t>
+  </si>
+  <si>
+    <t>67f68025cb21b80d2a91dc7b8444421c</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.7a8af6aa7044023ec038bd95b1fe4c0d3018c0328514b38734963865a0a2248f.8ca3055ce1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>Serv. Trasfusione non previsto in lab.</t>
   </si>
 </sst>
 </file>
@@ -1019,7 +1256,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1044,8 +1281,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="25">
     <border>
       <left/>
       <right/>
@@ -1341,12 +1584,34 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1491,6 +1756,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1512,6 +1778,15 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2950,16 +3225,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W580"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
     <col min="2" max="2" width="46.85546875" customWidth="1"/>
     <col min="3" max="3" width="20.140625" customWidth="1"/>
-    <col min="4" max="4" width="63.85546875" customWidth="1"/>
+    <col min="4" max="4" width="57" customWidth="1"/>
     <col min="5" max="5" width="47.28515625" customWidth="1"/>
     <col min="6" max="8" width="33.140625" customWidth="1"/>
-    <col min="9" max="9" width="81.42578125" customWidth="1"/>
+    <col min="9" max="9" width="47.85546875" customWidth="1"/>
     <col min="10" max="10" width="27.140625" customWidth="1"/>
     <col min="11" max="18" width="36.42578125" customWidth="1"/>
     <col min="19" max="19" width="27.140625" customWidth="1"/>
@@ -2991,14 +3267,14 @@
       <c r="W1" s="9"/>
     </row>
     <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="58" t="s">
+      <c r="B2" s="58"/>
+      <c r="C2" s="59" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="57"/>
+      <c r="D2" s="58"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
@@ -3019,14 +3295,14 @@
       <c r="W2" s="9"/>
     </row>
     <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="65" t="s">
+      <c r="B3" s="61"/>
+      <c r="C3" s="66" t="s">
         <v>141</v>
       </c>
-      <c r="D3" s="57"/>
+      <c r="D3" s="58"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
@@ -3047,12 +3323,12 @@
       <c r="W3" s="9"/>
     </row>
     <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="61"/>
-      <c r="B4" s="62"/>
-      <c r="C4" s="65" t="s">
+      <c r="A4" s="62"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="66" t="s">
         <v>142</v>
       </c>
-      <c r="D4" s="57"/>
+      <c r="D4" s="58"/>
       <c r="E4" s="4"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -3074,12 +3350,12 @@
       <c r="W4" s="9"/>
     </row>
     <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="63"/>
-      <c r="B5" s="64"/>
-      <c r="C5" s="65" t="s">
+      <c r="A5" s="64"/>
+      <c r="B5" s="65"/>
+      <c r="C5" s="66" t="s">
         <v>143</v>
       </c>
-      <c r="D5" s="57"/>
+      <c r="D5" s="58"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -3100,8 +3376,8 @@
       <c r="W5" s="9"/>
     </row>
     <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="54"/>
-      <c r="B6" s="55"/>
+      <c r="A6" s="55"/>
+      <c r="B6" s="56"/>
       <c r="C6" s="10"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -3236,7 +3512,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="33">
         <v>31</v>
       </c>
@@ -3297,7 +3573,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="33">
         <v>39</v>
       </c>
@@ -3358,7 +3634,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="33">
         <v>47</v>
       </c>
@@ -3415,7 +3691,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="33">
         <v>76</v>
       </c>
@@ -3476,7 +3752,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="33">
         <v>78</v>
       </c>
@@ -3537,7 +3813,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33">
         <v>79</v>
       </c>
@@ -3598,7 +3874,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="33">
         <v>80</v>
       </c>
@@ -3659,7 +3935,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:23" s="53" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" s="53" customFormat="1" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="45">
         <v>81</v>
       </c>
@@ -3700,7 +3976,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="33">
         <v>83</v>
       </c>
@@ -3761,7 +4037,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="33">
         <v>84</v>
       </c>
@@ -3822,7 +4098,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="33">
         <v>85</v>
       </c>
@@ -3883,7 +4159,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="33">
         <v>86</v>
       </c>
@@ -3944,7 +4220,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="33">
         <v>87</v>
       </c>
@@ -4005,7 +4281,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="33">
         <v>88</v>
       </c>
@@ -4066,7 +4342,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="33">
         <v>89</v>
       </c>
@@ -4127,7 +4403,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="33">
         <v>90</v>
       </c>
@@ -4188,7 +4464,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="33">
         <v>91</v>
       </c>
@@ -4249,7 +4525,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="33">
         <v>92</v>
       </c>
@@ -4310,7 +4586,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="33">
         <v>93</v>
       </c>
@@ -4371,7 +4647,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33">
         <v>462</v>
       </c>
@@ -4432,7 +4708,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="33">
         <v>471</v>
       </c>
@@ -4479,7 +4755,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33">
         <v>472</v>
       </c>
@@ -4526,7 +4802,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33">
         <v>474</v>
       </c>
@@ -4587,347 +4863,972 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
-      <c r="M33" s="7"/>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
-      <c r="R33" s="7"/>
-      <c r="S33" s="7"/>
-      <c r="T33" s="7"/>
-      <c r="U33" s="8"/>
-      <c r="V33" s="2"/>
-      <c r="W33" s="9"/>
-    </row>
-    <row r="34" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F34" s="6"/>
-      <c r="G34" s="6"/>
-      <c r="H34" s="6"/>
-      <c r="I34" s="6"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
-      <c r="L34" s="7"/>
-      <c r="M34" s="7"/>
-      <c r="N34" s="7"/>
-      <c r="O34" s="7"/>
-      <c r="P34" s="7"/>
-      <c r="Q34" s="7"/>
-      <c r="R34" s="7"/>
-      <c r="S34" s="7"/>
-      <c r="T34" s="7"/>
-      <c r="U34" s="8"/>
-      <c r="V34" s="2"/>
-      <c r="W34" s="9"/>
-    </row>
-    <row r="35" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F35" s="6"/>
-      <c r="G35" s="6"/>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="7"/>
-      <c r="M35" s="7"/>
-      <c r="N35" s="7"/>
-      <c r="O35" s="7"/>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="7"/>
-      <c r="R35" s="7"/>
-      <c r="S35" s="7"/>
-      <c r="T35" s="7"/>
-      <c r="U35" s="8"/>
-      <c r="V35" s="2"/>
-      <c r="W35" s="9"/>
-    </row>
-    <row r="36" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F36" s="6"/>
-      <c r="G36" s="6"/>
-      <c r="H36" s="6"/>
-      <c r="I36" s="6"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7"/>
-      <c r="M36" s="7"/>
-      <c r="N36" s="7"/>
-      <c r="O36" s="7"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="7"/>
-      <c r="R36" s="7"/>
-      <c r="S36" s="7"/>
-      <c r="T36" s="7"/>
-      <c r="U36" s="8"/>
-      <c r="V36" s="2"/>
-      <c r="W36" s="9"/>
-    </row>
-    <row r="37" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F37" s="6"/>
-      <c r="G37" s="6"/>
-      <c r="H37" s="6"/>
-      <c r="I37" s="6"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
-      <c r="M37" s="7"/>
-      <c r="N37" s="7"/>
-      <c r="O37" s="7"/>
-      <c r="P37" s="7"/>
-      <c r="Q37" s="7"/>
-      <c r="R37" s="7"/>
-      <c r="S37" s="7"/>
-      <c r="T37" s="7"/>
-      <c r="U37" s="8"/>
-      <c r="V37" s="2"/>
-      <c r="W37" s="9"/>
-    </row>
-    <row r="38" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F38" s="6"/>
-      <c r="G38" s="6"/>
-      <c r="H38" s="6"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
-      <c r="M38" s="7"/>
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="7"/>
-      <c r="R38" s="7"/>
-      <c r="S38" s="7"/>
-      <c r="T38" s="7"/>
-      <c r="U38" s="8"/>
-      <c r="V38" s="2"/>
-      <c r="W38" s="9"/>
-    </row>
-    <row r="39" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F39" s="6"/>
-      <c r="G39" s="6"/>
-      <c r="H39" s="6"/>
-      <c r="I39" s="6"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
-      <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="7"/>
-      <c r="P39" s="7"/>
-      <c r="Q39" s="7"/>
-      <c r="R39" s="7"/>
-      <c r="S39" s="7"/>
-      <c r="T39" s="7"/>
-      <c r="U39" s="8"/>
-      <c r="V39" s="2"/>
-      <c r="W39" s="9"/>
-    </row>
-    <row r="40" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F40" s="6"/>
-      <c r="G40" s="6"/>
-      <c r="H40" s="6"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
-      <c r="L40" s="7"/>
-      <c r="M40" s="7"/>
-      <c r="N40" s="7"/>
-      <c r="O40" s="7"/>
-      <c r="P40" s="7"/>
-      <c r="Q40" s="7"/>
-      <c r="R40" s="7"/>
-      <c r="S40" s="7"/>
-      <c r="T40" s="7"/>
-      <c r="U40" s="8"/>
-      <c r="V40" s="2"/>
-      <c r="W40" s="9"/>
-    </row>
-    <row r="41" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F41" s="6"/>
-      <c r="G41" s="6"/>
-      <c r="H41" s="6"/>
-      <c r="I41" s="6"/>
-      <c r="J41" s="7"/>
-      <c r="K41" s="7"/>
-      <c r="L41" s="7"/>
-      <c r="M41" s="7"/>
-      <c r="N41" s="7"/>
-      <c r="O41" s="7"/>
-      <c r="P41" s="7"/>
-      <c r="Q41" s="7"/>
-      <c r="R41" s="7"/>
-      <c r="S41" s="7"/>
-      <c r="T41" s="7"/>
-      <c r="U41" s="8"/>
-      <c r="V41" s="2"/>
-      <c r="W41" s="9"/>
-    </row>
-    <row r="42" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F42" s="6"/>
-      <c r="G42" s="6"/>
-      <c r="H42" s="6"/>
-      <c r="I42" s="6"/>
-      <c r="J42" s="7"/>
-      <c r="K42" s="7"/>
-      <c r="L42" s="7"/>
-      <c r="M42" s="7"/>
-      <c r="N42" s="7"/>
-      <c r="O42" s="7"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="7"/>
-      <c r="R42" s="7"/>
-      <c r="S42" s="7"/>
-      <c r="T42" s="7"/>
-      <c r="U42" s="8"/>
-      <c r="V42" s="2"/>
-      <c r="W42" s="9"/>
-    </row>
-    <row r="43" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="7"/>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="7"/>
-      <c r="P43" s="7"/>
-      <c r="Q43" s="7"/>
-      <c r="R43" s="7"/>
-      <c r="S43" s="7"/>
-      <c r="T43" s="7"/>
-      <c r="U43" s="8"/>
-      <c r="V43" s="2"/>
-      <c r="W43" s="9"/>
-    </row>
-    <row r="44" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F44" s="6"/>
-      <c r="G44" s="6"/>
-      <c r="H44" s="6"/>
-      <c r="I44" s="6"/>
-      <c r="J44" s="7"/>
-      <c r="K44" s="7"/>
-      <c r="L44" s="7"/>
-      <c r="M44" s="7"/>
-      <c r="N44" s="7"/>
-      <c r="O44" s="7"/>
-      <c r="P44" s="7"/>
-      <c r="Q44" s="7"/>
-      <c r="R44" s="7"/>
-      <c r="S44" s="7"/>
-      <c r="T44" s="7"/>
-      <c r="U44" s="8"/>
-      <c r="V44" s="2"/>
-      <c r="W44" s="9"/>
-    </row>
-    <row r="45" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F45" s="6"/>
-      <c r="G45" s="6"/>
-      <c r="H45" s="6"/>
-      <c r="I45" s="6"/>
-      <c r="J45" s="7"/>
-      <c r="K45" s="7"/>
-      <c r="L45" s="7"/>
-      <c r="M45" s="7"/>
-      <c r="N45" s="7"/>
-      <c r="O45" s="7"/>
-      <c r="P45" s="7"/>
-      <c r="Q45" s="7"/>
-      <c r="R45" s="7"/>
-      <c r="S45" s="7"/>
-      <c r="T45" s="7"/>
-      <c r="U45" s="8"/>
-      <c r="V45" s="2"/>
-      <c r="W45" s="9"/>
-    </row>
-    <row r="46" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F46" s="6"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="6"/>
-      <c r="I46" s="6"/>
-      <c r="J46" s="7"/>
-      <c r="K46" s="7"/>
-      <c r="L46" s="7"/>
-      <c r="M46" s="7"/>
-      <c r="N46" s="7"/>
-      <c r="O46" s="7"/>
-      <c r="P46" s="7"/>
-      <c r="Q46" s="7"/>
-      <c r="R46" s="7"/>
-      <c r="S46" s="7"/>
-      <c r="T46" s="7"/>
-      <c r="U46" s="8"/>
-      <c r="V46" s="2"/>
-      <c r="W46" s="9"/>
-    </row>
-    <row r="47" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F47" s="6"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="6"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="7"/>
-      <c r="K47" s="7"/>
-      <c r="L47" s="7"/>
-      <c r="M47" s="7"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="7"/>
-      <c r="P47" s="7"/>
-      <c r="Q47" s="7"/>
-      <c r="R47" s="7"/>
-      <c r="S47" s="7"/>
-      <c r="T47" s="7"/>
-      <c r="U47" s="8"/>
-      <c r="V47" s="2"/>
-      <c r="W47" s="9"/>
-    </row>
-    <row r="48" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F48" s="6"/>
-      <c r="G48" s="6"/>
-      <c r="H48" s="6"/>
-      <c r="I48" s="6"/>
-      <c r="J48" s="7"/>
-      <c r="K48" s="7"/>
-      <c r="L48" s="7"/>
-      <c r="M48" s="7"/>
-      <c r="N48" s="7"/>
-      <c r="O48" s="7"/>
-      <c r="P48" s="7"/>
-      <c r="Q48" s="7"/>
-      <c r="R48" s="7"/>
-      <c r="S48" s="7"/>
-      <c r="T48" s="7"/>
-      <c r="U48" s="8"/>
-      <c r="V48" s="2"/>
-      <c r="W48" s="9"/>
-    </row>
-    <row r="49" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F49" s="6"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="6"/>
-      <c r="I49" s="6"/>
-      <c r="J49" s="7"/>
-      <c r="K49" s="7"/>
-      <c r="L49" s="7"/>
-      <c r="M49" s="7"/>
-      <c r="N49" s="7"/>
-      <c r="O49" s="7"/>
-      <c r="P49" s="7"/>
-      <c r="Q49" s="7"/>
-      <c r="R49" s="7"/>
-      <c r="S49" s="7"/>
-      <c r="T49" s="7"/>
-      <c r="U49" s="8"/>
-      <c r="V49" s="2"/>
-      <c r="W49" s="9"/>
-    </row>
-    <row r="50" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="67">
+        <v>4</v>
+      </c>
+      <c r="B33" s="67" t="s">
+        <v>34</v>
+      </c>
+      <c r="C33" s="68" t="s">
+        <v>35</v>
+      </c>
+      <c r="D33" s="69" t="s">
+        <v>211</v>
+      </c>
+      <c r="E33" s="40" t="s">
+        <v>212</v>
+      </c>
+      <c r="F33" s="34">
+        <v>46235</v>
+      </c>
+      <c r="G33" s="34" t="s">
+        <v>243</v>
+      </c>
+      <c r="H33" s="34" t="s">
+        <v>242</v>
+      </c>
+      <c r="I33" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="J33" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K33" s="35"/>
+      <c r="L33" s="35"/>
+      <c r="M33" s="35"/>
+      <c r="N33" s="35"/>
+      <c r="O33" s="35"/>
+      <c r="P33" s="35"/>
+      <c r="Q33" s="35"/>
+      <c r="R33" s="35"/>
+      <c r="S33" s="35"/>
+      <c r="T33" s="35"/>
+      <c r="U33" s="36"/>
+      <c r="V33" s="37"/>
+      <c r="W33" s="35" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="33">
+        <v>28</v>
+      </c>
+      <c r="B34" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D34" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="E34" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F34" s="34">
+        <v>46235</v>
+      </c>
+      <c r="G34" s="34" t="s">
+        <v>247</v>
+      </c>
+      <c r="H34" s="34" t="s">
+        <v>248</v>
+      </c>
+      <c r="I34" s="39" t="s">
+        <v>198</v>
+      </c>
+      <c r="J34" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K34" s="35"/>
+      <c r="L34" s="35"/>
+      <c r="M34" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N34" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O34" s="35" t="s">
+        <v>201</v>
+      </c>
+      <c r="P34" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q34" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R34" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S34" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="T34" s="35"/>
+      <c r="U34" s="36"/>
+      <c r="V34" s="37"/>
+      <c r="W34" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="33">
+        <v>36</v>
+      </c>
+      <c r="B35" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C35" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D35" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="E35" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F35" s="34">
+        <v>46235</v>
+      </c>
+      <c r="G35" s="34" t="s">
+        <v>245</v>
+      </c>
+      <c r="H35" s="34" t="s">
+        <v>246</v>
+      </c>
+      <c r="I35" s="39" t="s">
+        <v>198</v>
+      </c>
+      <c r="J35" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K35" s="35"/>
+      <c r="L35" s="35"/>
+      <c r="M35" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N35" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O35" s="35" t="s">
+        <v>201</v>
+      </c>
+      <c r="P35" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q35" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R35" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S35" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="T35" s="35"/>
+      <c r="U35" s="36"/>
+      <c r="V35" s="37"/>
+      <c r="W35" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="33">
+        <v>44</v>
+      </c>
+      <c r="B36" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D36" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="E36" s="40" t="s">
+        <v>133</v>
+      </c>
+      <c r="F36" s="34">
+        <v>46235</v>
+      </c>
+      <c r="G36" s="34" t="s">
+        <v>249</v>
+      </c>
+      <c r="H36" s="34"/>
+      <c r="I36" s="39"/>
+      <c r="J36" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K36" s="35"/>
+      <c r="L36" s="35"/>
+      <c r="M36" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N36" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O36" s="35" t="s">
+        <v>195</v>
+      </c>
+      <c r="P36" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q36" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R36" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S36" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="T36" s="35"/>
+      <c r="U36" s="36"/>
+      <c r="V36" s="37"/>
+      <c r="W36" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="33">
+        <v>53</v>
+      </c>
+      <c r="B37" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D37" s="33" t="s">
+        <v>216</v>
+      </c>
+      <c r="E37" s="40" t="s">
+        <v>217</v>
+      </c>
+      <c r="F37" s="34">
+        <v>46235</v>
+      </c>
+      <c r="G37" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="H37" s="34" t="s">
+        <v>253</v>
+      </c>
+      <c r="I37" s="39" t="s">
+        <v>255</v>
+      </c>
+      <c r="J37" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K37" s="35"/>
+      <c r="L37" s="35"/>
+      <c r="M37" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N37" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O37" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P37" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q37" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R37" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S37" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T37" s="35"/>
+      <c r="U37" s="36"/>
+      <c r="V37" s="37"/>
+      <c r="W37" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="33">
+        <v>55</v>
+      </c>
+      <c r="B38" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C38" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D38" s="33" t="s">
+        <v>218</v>
+      </c>
+      <c r="E38" s="40" t="s">
+        <v>219</v>
+      </c>
+      <c r="F38" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G38" s="34" t="s">
+        <v>257</v>
+      </c>
+      <c r="H38" s="34" t="s">
+        <v>256</v>
+      </c>
+      <c r="I38" s="39" t="s">
+        <v>258</v>
+      </c>
+      <c r="J38" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K38" s="35"/>
+      <c r="L38" s="35"/>
+      <c r="M38" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N38" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O38" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P38" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q38" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R38" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S38" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T38" s="35"/>
+      <c r="U38" s="36"/>
+      <c r="V38" s="37"/>
+      <c r="W38" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="33">
+        <v>56</v>
+      </c>
+      <c r="B39" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D39" s="33" t="s">
+        <v>220</v>
+      </c>
+      <c r="E39" s="40" t="s">
+        <v>221</v>
+      </c>
+      <c r="F39" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G39" s="34" t="s">
+        <v>260</v>
+      </c>
+      <c r="H39" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="I39" s="39" t="s">
+        <v>261</v>
+      </c>
+      <c r="J39" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K39" s="35"/>
+      <c r="L39" s="35"/>
+      <c r="M39" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N39" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O39" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P39" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q39" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R39" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S39" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T39" s="35"/>
+      <c r="U39" s="36"/>
+      <c r="V39" s="37"/>
+      <c r="W39" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="33">
+        <v>57</v>
+      </c>
+      <c r="B40" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C40" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="E40" s="40" t="s">
+        <v>223</v>
+      </c>
+      <c r="F40" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G40" s="34" t="s">
+        <v>263</v>
+      </c>
+      <c r="H40" s="34" t="s">
+        <v>262</v>
+      </c>
+      <c r="I40" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="J40" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K40" s="35"/>
+      <c r="L40" s="35"/>
+      <c r="M40" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N40" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O40" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P40" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q40" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R40" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S40" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T40" s="35"/>
+      <c r="U40" s="36"/>
+      <c r="V40" s="37"/>
+      <c r="W40" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="33">
+        <v>59</v>
+      </c>
+      <c r="B41" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C41" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D41" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="E41" s="40" t="s">
+        <v>225</v>
+      </c>
+      <c r="F41" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G41" s="34" t="s">
+        <v>267</v>
+      </c>
+      <c r="H41" s="34" t="s">
+        <v>265</v>
+      </c>
+      <c r="I41" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="J41" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K41" s="35"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N41" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O41" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P41" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q41" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R41" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S41" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T41" s="35"/>
+      <c r="U41" s="36"/>
+      <c r="V41" s="37"/>
+      <c r="W41" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="33">
+        <v>60</v>
+      </c>
+      <c r="B42" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C42" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="33" t="s">
+        <v>226</v>
+      </c>
+      <c r="E42" s="40" t="s">
+        <v>227</v>
+      </c>
+      <c r="F42" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G42" s="34" t="s">
+        <v>269</v>
+      </c>
+      <c r="H42" s="34" t="s">
+        <v>268</v>
+      </c>
+      <c r="I42" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="J42" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K42" s="35"/>
+      <c r="L42" s="35"/>
+      <c r="M42" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N42" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O42" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P42" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q42" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R42" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S42" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T42" s="35"/>
+      <c r="U42" s="36"/>
+      <c r="V42" s="37"/>
+      <c r="W42" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="33">
+        <v>61</v>
+      </c>
+      <c r="B43" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C43" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D43" s="33" t="s">
+        <v>228</v>
+      </c>
+      <c r="E43" s="40" t="s">
+        <v>229</v>
+      </c>
+      <c r="F43" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G43" s="34" t="s">
+        <v>273</v>
+      </c>
+      <c r="H43" s="34" t="s">
+        <v>271</v>
+      </c>
+      <c r="I43" s="39" t="s">
+        <v>272</v>
+      </c>
+      <c r="J43" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K43" s="35"/>
+      <c r="L43" s="35"/>
+      <c r="M43" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N43" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O43" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P43" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q43" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R43" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S43" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T43" s="35"/>
+      <c r="U43" s="36"/>
+      <c r="V43" s="37"/>
+      <c r="W43" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="33">
+        <v>62</v>
+      </c>
+      <c r="B44" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C44" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D44" s="33" t="s">
+        <v>230</v>
+      </c>
+      <c r="E44" s="40" t="s">
+        <v>231</v>
+      </c>
+      <c r="F44" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G44" s="34" t="s">
+        <v>280</v>
+      </c>
+      <c r="H44" s="34" t="s">
+        <v>281</v>
+      </c>
+      <c r="I44" s="39" t="s">
+        <v>282</v>
+      </c>
+      <c r="J44" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K44" s="35"/>
+      <c r="L44" s="35"/>
+      <c r="M44" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N44" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O44" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P44" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q44" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R44" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S44" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T44" s="35"/>
+      <c r="U44" s="36"/>
+      <c r="V44" s="37"/>
+      <c r="W44" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" s="54" customFormat="1" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="33">
+        <v>191</v>
+      </c>
+      <c r="B45" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C45" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D45" s="33" t="s">
+        <v>232</v>
+      </c>
+      <c r="E45" s="40" t="s">
+        <v>233</v>
+      </c>
+      <c r="F45" s="34"/>
+      <c r="G45" s="34"/>
+      <c r="H45" s="34"/>
+      <c r="I45" s="39"/>
+      <c r="J45" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="K45" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="L45" s="35" t="s">
+        <v>283</v>
+      </c>
+      <c r="M45" s="35"/>
+      <c r="N45" s="35"/>
+      <c r="O45" s="35"/>
+      <c r="P45" s="35"/>
+      <c r="Q45" s="35"/>
+      <c r="R45" s="35"/>
+      <c r="S45" s="35"/>
+      <c r="T45" s="35"/>
+      <c r="U45" s="36"/>
+      <c r="V45" s="37"/>
+      <c r="W45" s="35"/>
+    </row>
+    <row r="46" spans="1:23" s="54" customFormat="1" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="33">
+        <v>376</v>
+      </c>
+      <c r="B46" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C46" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D46" s="33" t="s">
+        <v>234</v>
+      </c>
+      <c r="E46" s="40" t="s">
+        <v>235</v>
+      </c>
+      <c r="F46" s="34"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="34"/>
+      <c r="I46" s="39"/>
+      <c r="J46" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="K46" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="L46" s="35" t="s">
+        <v>283</v>
+      </c>
+      <c r="M46" s="35"/>
+      <c r="N46" s="35"/>
+      <c r="O46" s="35"/>
+      <c r="P46" s="35"/>
+      <c r="Q46" s="35"/>
+      <c r="R46" s="35"/>
+      <c r="S46" s="35"/>
+      <c r="T46" s="35"/>
+      <c r="U46" s="36"/>
+      <c r="V46" s="37"/>
+      <c r="W46" s="35"/>
+    </row>
+    <row r="47" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="33">
+        <v>452</v>
+      </c>
+      <c r="B47" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C47" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D47" s="69" t="s">
+        <v>236</v>
+      </c>
+      <c r="E47" s="40" t="s">
+        <v>237</v>
+      </c>
+      <c r="F47" s="34">
+        <v>46235</v>
+      </c>
+      <c r="G47" s="34" t="s">
+        <v>250</v>
+      </c>
+      <c r="H47" s="34" t="s">
+        <v>251</v>
+      </c>
+      <c r="I47" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="J47" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K47" s="35"/>
+      <c r="L47" s="35"/>
+      <c r="M47" s="35"/>
+      <c r="N47" s="35"/>
+      <c r="O47" s="35"/>
+      <c r="P47" s="35"/>
+      <c r="Q47" s="35"/>
+      <c r="R47" s="35"/>
+      <c r="S47" s="35"/>
+      <c r="T47" s="35"/>
+      <c r="U47" s="36"/>
+      <c r="V47" s="37"/>
+      <c r="W47" s="35" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="33">
+        <v>466</v>
+      </c>
+      <c r="B48" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C48" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D48" s="33" t="s">
+        <v>238</v>
+      </c>
+      <c r="E48" s="40" t="s">
+        <v>239</v>
+      </c>
+      <c r="F48" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G48" s="34" t="s">
+        <v>276</v>
+      </c>
+      <c r="H48" s="34" t="s">
+        <v>275</v>
+      </c>
+      <c r="I48" s="39" t="s">
+        <v>274</v>
+      </c>
+      <c r="J48" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K48" s="35"/>
+      <c r="L48" s="35"/>
+      <c r="M48" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N48" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O48" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P48" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q48" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R48" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S48" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T48" s="35"/>
+      <c r="U48" s="36"/>
+      <c r="V48" s="37"/>
+      <c r="W48" s="33" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" s="54" customFormat="1" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="33">
+        <v>473</v>
+      </c>
+      <c r="B49" s="33" t="s">
+        <v>34</v>
+      </c>
+      <c r="C49" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="D49" s="38" t="s">
+        <v>240</v>
+      </c>
+      <c r="E49" s="40" t="s">
+        <v>241</v>
+      </c>
+      <c r="F49" s="34">
+        <v>46236</v>
+      </c>
+      <c r="G49" s="34" t="s">
+        <v>279</v>
+      </c>
+      <c r="H49" s="34" t="s">
+        <v>277</v>
+      </c>
+      <c r="I49" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="J49" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="K49" s="35"/>
+      <c r="L49" s="35"/>
+      <c r="M49" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="N49" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="O49" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="P49" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q49" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="R49" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="S49" s="35" t="s">
+        <v>148</v>
+      </c>
+      <c r="T49" s="35"/>
+      <c r="U49" s="36"/>
+      <c r="V49" s="37"/>
+      <c r="W49" s="35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F50" s="6"/>
       <c r="G50" s="6"/>
       <c r="H50" s="6"/>
@@ -4947,7 +5848,7 @@
       <c r="V50" s="2"/>
       <c r="W50" s="9"/>
     </row>
-    <row r="51" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
@@ -4967,7 +5868,7 @@
       <c r="V51" s="2"/>
       <c r="W51" s="9"/>
     </row>
-    <row r="52" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
@@ -4987,7 +5888,7 @@
       <c r="V52" s="2"/>
       <c r="W52" s="9"/>
     </row>
-    <row r="53" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -5007,7 +5908,7 @@
       <c r="V53" s="2"/>
       <c r="W53" s="9"/>
     </row>
-    <row r="54" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -5027,7 +5928,7 @@
       <c r="V54" s="2"/>
       <c r="W54" s="9"/>
     </row>
-    <row r="55" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>
@@ -5047,7 +5948,7 @@
       <c r="V55" s="2"/>
       <c r="W55" s="9"/>
     </row>
-    <row r="56" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>
@@ -5067,7 +5968,7 @@
       <c r="V56" s="2"/>
       <c r="W56" s="9"/>
     </row>
-    <row r="57" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F57" s="6"/>
       <c r="G57" s="6"/>
       <c r="H57" s="6"/>
@@ -5087,7 +5988,7 @@
       <c r="V57" s="2"/>
       <c r="W57" s="9"/>
     </row>
-    <row r="58" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F58" s="6"/>
       <c r="G58" s="6"/>
       <c r="H58" s="6"/>
@@ -5107,7 +6008,7 @@
       <c r="V58" s="2"/>
       <c r="W58" s="9"/>
     </row>
-    <row r="59" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
       <c r="H59" s="6"/>
@@ -5127,7 +6028,7 @@
       <c r="V59" s="2"/>
       <c r="W59" s="9"/>
     </row>
-    <row r="60" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F60" s="6"/>
       <c r="G60" s="6"/>
       <c r="H60" s="6"/>
@@ -5147,7 +6048,7 @@
       <c r="V60" s="2"/>
       <c r="W60" s="9"/>
     </row>
-    <row r="61" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F61" s="6"/>
       <c r="G61" s="6"/>
       <c r="H61" s="6"/>
@@ -5167,7 +6068,7 @@
       <c r="V61" s="2"/>
       <c r="W61" s="9"/>
     </row>
-    <row r="62" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F62" s="6"/>
       <c r="G62" s="6"/>
       <c r="H62" s="6"/>
@@ -5187,7 +6088,7 @@
       <c r="V62" s="2"/>
       <c r="W62" s="9"/>
     </row>
-    <row r="63" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F63" s="6"/>
       <c r="G63" s="6"/>
       <c r="H63" s="6"/>
@@ -5207,7 +6108,7 @@
       <c r="V63" s="2"/>
       <c r="W63" s="9"/>
     </row>
-    <row r="64" spans="6:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F64" s="6"/>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
@@ -8364,7 +9265,13 @@
     <row r="579" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="580" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A9:W32" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <autoFilter ref="A9:W49" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="LAB"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="7">
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A2:B2"/>
@@ -8385,19 +9292,19 @@
           <x14:formula1>
             <xm:f>Sheet1!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J10:J32 M10:N32 P10:R32</xm:sqref>
+          <xm:sqref>M47:N49 J10:J49 M10:N44 P10:R44 P47:R49</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showErrorMessage="1" xr:uid="{70793024-27E9-4E6A-BACD-083AB683BC38}">
           <x14:formula1>
             <xm:f>Sheet1!$A$2:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>T10:T32</xm:sqref>
+          <xm:sqref>T10:T44 T47:T49</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3DE61C5E-9DA3-4CE3-A1FF-8FBE651EA6B5}">
           <x14:formula1>
             <xm:f>'LISTA VALORI'!$A$2:$A$8</xm:f>
           </x14:formula1>
-          <xm:sqref>K10:K32</xm:sqref>
+          <xm:sqref>K10:K49</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -10634,6 +11541,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100BE9A258ADBC3EC4CBEB1E2AB9909207A" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0284f501378927579289f00316ec8a74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="295b7897-c886-40bf-9750-5782b814c3e4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b47213d65be806e283915cff374a7eef" ns2:_="">
     <xsd:import namespace="295b7897-c886-40bf-9750-5782b814c3e4"/>
@@ -10777,35 +11699,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="295b7897-c886-40bf-9750-5782b814c3e4"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10828,9 +11725,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7568E770-0BC4-46AF-B6C6-958AE21C8F7F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="295b7897-c886-40bf-9750-5782b814c3e4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>